<commit_message>
QA G1: actualización de la bitácora de pruebas
</commit_message>
<xml_diff>
--- a/grupos/grupo-1-base-de-datos/qa/BITACORA BASES DE DATOS.xlsx
+++ b/grupos/grupo-1-base-de-datos/qa/BITACORA BASES DE DATOS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Example\Documents\Ingenieria en Sistemas Ang\4 Semestre\PROGRAMACIÓN WEB\APLICACIÓN PROYECTO\BASE DE DATOS - GRUPO 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Example\Documents\Ingenieria en Sistemas Ang\4 Semestre\PROGRAMACIÓN WEB\APLICACIÓN PROYECTO\BASE DE DATOS - GRUPO 1\QA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F57D470-91D4-457A-A043-C789CB483BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D13C2C-3601-4B26-A51E-5FF6C1078112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="45" windowWidth="21060" windowHeight="15585" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bases de datos" sheetId="3" r:id="rId1"/>
@@ -423,7 +423,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="390">
   <si>
     <t>Automatización</t>
   </si>
@@ -1441,9 +1441,6 @@
   </si>
   <si>
     <t>Medio</t>
-  </si>
-  <si>
-    <t>Nuevo</t>
   </si>
   <si>
     <t>Angel Aguilar</t>
@@ -1761,6 +1758,31 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
         <name val="Arial"/>
         <charset val="1"/>
@@ -1780,31 +1802,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2451,7 +2448,7 @@
         <v>326</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>11</v>
@@ -2471,7 +2468,7 @@
         <v>328</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>15</v>
@@ -2534,7 +2531,9 @@
       <c r="K6" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="L6" s="4"/>
+      <c r="L6" s="5">
+        <v>46300</v>
+      </c>
       <c r="M6" s="4"/>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -2573,12 +2572,14 @@
       <c r="K7" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="L7" s="4"/>
+      <c r="L7" s="5">
+        <v>46300</v>
+      </c>
       <c r="M7" s="4" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="O7" s="4"/>
     </row>
@@ -2834,7 +2835,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="O13" s="4"/>
     </row>
@@ -2879,7 +2880,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>334</v>
@@ -2926,7 +2927,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N15" s="4" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="O15" s="4"/>
     </row>
@@ -2971,7 +2972,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="O16" s="4"/>
     </row>
@@ -3016,7 +3017,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="O17" s="4"/>
     </row>
@@ -3061,7 +3062,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="O18" s="4"/>
     </row>
@@ -3104,7 +3105,7 @@
       </c>
       <c r="M19" s="4"/>
       <c r="N19" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="O19" s="4"/>
     </row>
@@ -3192,7 +3193,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N21" s="4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="O21" s="4"/>
     </row>
@@ -3237,7 +3238,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N22" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="O22" s="4"/>
     </row>
@@ -3282,7 +3283,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N23" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="O23" s="4"/>
     </row>
@@ -3327,7 +3328,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O24" s="4"/>
     </row>
@@ -3372,7 +3373,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="O25" s="4"/>
     </row>
@@ -3417,7 +3418,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O26" s="4"/>
     </row>
@@ -3479,7 +3480,7 @@
         <v>132</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>56</v>
@@ -3503,10 +3504,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="1:15" ht="39.6" x14ac:dyDescent="0.3">
@@ -3591,7 +3592,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N30" s="4" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="O30" s="6"/>
     </row>
@@ -3677,7 +3678,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N32" s="4" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="O32" s="6"/>
     </row>
@@ -3739,7 +3740,7 @@
         <v>161</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>56</v>
@@ -3763,10 +3764,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="N34" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="35" spans="1:15" ht="59.4" x14ac:dyDescent="0.3">
@@ -3851,7 +3852,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N36" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="O36" s="4"/>
     </row>
@@ -3894,7 +3895,7 @@
       </c>
       <c r="M37" s="4"/>
       <c r="N37" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="O37" s="4"/>
     </row>
@@ -3939,7 +3940,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N38" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O38" s="4"/>
     </row>
@@ -4109,10 +4110,10 @@
         <v>#VALUE!</v>
       </c>
       <c r="N42" s="4" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="43" spans="1:15" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
@@ -4156,7 +4157,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N43" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="O43" s="4"/>
     </row>
@@ -4201,7 +4202,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N44" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="O44" s="4"/>
     </row>
@@ -4578,7 +4579,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N53" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="O53" s="4"/>
     </row>
@@ -4664,7 +4665,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N55" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="O55" s="4"/>
     </row>
@@ -4709,7 +4710,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="N56" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="O56" s="4"/>
     </row>
@@ -4751,7 +4752,7 @@
         <v>46316</v>
       </c>
       <c r="M57" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="N57" s="4"/>
       <c r="O57" s="4"/>
@@ -4794,7 +4795,7 @@
         <v>46317</v>
       </c>
       <c r="M58" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="N58" s="4"/>
       <c r="O58" s="4"/>
@@ -5052,13 +5053,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="J5:J303">
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$J5="Pasó"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$J5="Falló"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$J5="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5159,7 +5160,7 @@
         <v>322</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>63</v>
@@ -5183,10 +5184,10 @@
         <v>17</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="N2" s="7" t="e" vm="34">
         <v>#VALUE!</v>
@@ -5195,12 +5196,12 @@
         <v>46306</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="115.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B3" s="8">
         <v>46302</v>
@@ -5209,7 +5210,7 @@
         <v>322</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>129</v>
@@ -5218,13 +5219,13 @@
         <v>124</v>
       </c>
       <c r="G3" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>345</v>
-      </c>
-      <c r="H3" s="7" t="s">
-        <v>347</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>346</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>338</v>
@@ -5233,10 +5234,10 @@
         <v>17</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="N3" s="4" t="e" vm="35">
         <v>#VALUE!</v>
@@ -5245,12 +5246,12 @@
         <v>46306</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B4" s="8">
         <v>46302</v>
@@ -5259,7 +5260,7 @@
         <v>322</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>158</v>
@@ -5268,25 +5269,25 @@
         <v>124</v>
       </c>
       <c r="G4" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="I4" s="7" t="s">
         <v>351</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="J4" s="7" t="s">
         <v>353</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>352</v>
-      </c>
-      <c r="J4" s="7" t="s">
-        <v>354</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="N4" s="4" t="e" vm="36">
         <v>#VALUE!</v>
@@ -5295,12 +5296,12 @@
         <v>46306</v>
       </c>
       <c r="P4" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="162" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B5" s="8">
         <v>46302</v>
@@ -5309,7 +5310,7 @@
         <v>322</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>195</v>
@@ -5318,25 +5319,25 @@
         <v>196</v>
       </c>
       <c r="G5" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="H5" s="7" t="s">
         <v>356</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>357</v>
       </c>
-      <c r="I5" s="7" t="s">
-        <v>358</v>
-      </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="7" t="s">
         <v>338</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>17</v>
       </c>
       <c r="L5" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="M5" s="7" t="s">
         <v>339</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>340</v>
       </c>
       <c r="N5" s="4" t="e" vm="37">
         <v>#VALUE!</v>
@@ -5345,7 +5346,7 @@
         <v>46306</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -10662,10 +10663,10 @@
   <autoFilter ref="A1:P300" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="J2:J300">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>$J2="Crítico"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>$J2="Alto"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>